<commit_message>
Add break-even and payment sensitivity figures, table 8, and log entry
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/capabilities/economic-research/model.xlsx
+++ b/capabilities/economic-research/model.xlsx
@@ -297,6 +297,530 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Rise in local visitors needed to break even (90-day campaign)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>$1 gift shop</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$68:$B$72</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$D$68:$D$72</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>$2.5 gift shop</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$68:$B$72</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$E$68:$E$72</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>$5 gift shop</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$68:$B$72</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$F$68:$F$72</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>$7.5 gift shop</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$68:$B$72</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$G$68:$G$72</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <v>$10 gift shop</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$68:$B$72</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$H$68:$H$72</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <v>$15 gift shop</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$68:$B$72</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$I$68:$I$72</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Marketing spend</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Rise in today's local visitors</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Rise in local visitors needed vs. average PWYW payment</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>$5,000 marketing</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$77:$B$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$C$77:$C$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>$10,000 marketing</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$77:$B$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$D$77:$D$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>$15,000 marketing</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$77:$B$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$E$77:$E$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>$20,000 marketing</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sensitivity'!$B$77:$B$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sensitivity'!$F$77:$F$87</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Campaign-average payment ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Rise in today's local visitors</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>54</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3420000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>74</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3420000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2124,7 +2648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I72"/>
+  <dimension ref="B2:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3741,6 +4265,274 @@
       <c r="I72" s="14">
         <f>IF(ISNUMBER(IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*Average_PWYW-Headset_Cost)+I$66)&lt;=0,"n/a",($B72/Campaign_Days-Locals_Base*(1-EXP(-$B72/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*Average_PWYW-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*Average_PWYW-Headset_Cost)+I$66))),IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*Average_PWYW-Headset_Cost)+I$66)&lt;=0,"n/a",($B72/Campaign_Days-Locals_Base*(1-EXP(-$B72/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*Average_PWYW-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*Average_PWYW-Headset_Cost)+I$66))/Locals_Base,"n/a")</f>
         <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>8. BREAK-EVEN rise in local visitors vs. campaign-average payment (base gift shop spend)</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="n"/>
+      <c r="D75" s="5" t="n"/>
+      <c r="E75" s="5" t="n"/>
+      <c r="F75" s="5" t="n"/>
+    </row>
+    <row r="76">
+      <c r="B76" s="24" t="inlineStr">
+        <is>
+          <t>Avg payment ($) \ Marketing ($)</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D76" s="11" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E76" s="11" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F76" s="11" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B77-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B77-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B77-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D77" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B77-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B77-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B77-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E77" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B77-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B77-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B77-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F77" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B77-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B77-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B77-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B78-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B78-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B78-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D78" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B78-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B78-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B78-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E78" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B78-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B78-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B78-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F78" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B78-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B78-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B78-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B79-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B79-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B79-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D79" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B79-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B79-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B79-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E79" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B79-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B79-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B79-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F79" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B79-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B79-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B79-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C80" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B80-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B80-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B80-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D80" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B80-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B80-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B80-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E80" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B80-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B80-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B80-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F80" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B80-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B80-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B80-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C81" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B81-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B81-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B81-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D81" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B81-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B81-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B81-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E81" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B81-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B81-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B81-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F81" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B81-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B81-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B81-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C82" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B82-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B82-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B82-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D82" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B82-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B82-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B82-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E82" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B82-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B82-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B82-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F82" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B82-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B82-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B82-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C83" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B83-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B83-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B83-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D83" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B83-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B83-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B83-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E83" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B83-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B83-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B83-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F83" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B83-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B83-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B83-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C84" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B84-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B84-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B84-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D84" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B84-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B84-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B84-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E84" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B84-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B84-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B84-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F84" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B84-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B84-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B84-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C85" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B85-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B85-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B85-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D85" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B85-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B85-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B85-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E85" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B85-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B85-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B85-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F85" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B85-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B85-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B85-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C86" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B86-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B86-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B86-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D86" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B86-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B86-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B86-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E86" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B86-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B86-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B86-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F86" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B86-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B86-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B86-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C87" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B87-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((C$76/Campaign_Days-Locals_Base*(1-EXP(-C$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B87-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B87-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="D87" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B87-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((D$76/Campaign_Days-Locals_Base*(1-EXP(-D$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B87-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B87-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="E87" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B87-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((E$76/Campaign_Days-Locals_Base*(1-EXP(-E$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B87-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B87-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+      <c r="F87" s="14">
+        <f>IF((Local_AudioTour_Rate_PWYW*(Fee_Keep*$B87-Headset_Cost)+GiftShop_Net_Spend_Local)&lt;=0,"n/a",((F$76/Campaign_Days-Locals_Base*(1-EXP(-F$76/Marketing_Saturation_Spend))*(Fee_Keep*(Local_AudioTour_Rate_PWYW*$B87-Local_AudioTour_Rate_Init*AudioTour_Price)-Headset_Cost*(Local_AudioTour_Rate_PWYW-Local_AudioTour_Rate_Init)+Local_AudioTour_Rate_PWYW*GiftShop_Spillover))/(Local_AudioTour_Rate_PWYW*(Fee_Keep*$B87-Headset_Cost)+GiftShop_Net_Spend_Local))/Locals_Base)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Negative = the program pays for itself with no added locals (existing locals paying more than $7 cover the campaign). Compare with the campaign-average payment of the base case on the Model tab.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3785,6 +4577,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>